<commit_message>
Upload Data Analysis Spreadsheet
</commit_message>
<xml_diff>
--- a/Primitive Testing Data Analysis.xlsx
+++ b/Primitive Testing Data Analysis.xlsx
@@ -8,16 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lfam/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A13360B4-38D2-4242-A873-8C23F8D13350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49250426-0583-BC47-99DE-A593878AE588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="1740" windowWidth="27240" windowHeight="15980" xr2:uid="{9D05CCF2-C429-884D-8DA9-DCC0300FE582}"/>
+    <workbookView xWindow="20" yWindow="1740" windowWidth="22120" windowHeight="15980" xr2:uid="{9D05CCF2-C429-884D-8DA9-DCC0300FE582}"/>
   </bookViews>
   <sheets>
-    <sheet name="crypto_results_death (2)" sheetId="1" r:id="rId1"/>
+    <sheet name="Data Analysis" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'crypto_results_death (2)'!$B$1:$X$23</definedName>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'crypto_results_death (2)'!$B$1:$X$23</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">'Data Analysis'!$AB$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Data Analysis'!$AB$2:$AB$23</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Data Analysis'!$Y$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Data Analysis'!$Y$2:$Y$23</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'Data Analysis'!$AF$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'Data Analysis'!$AF$2:$AF$23</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'Data Analysis'!$AB$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">'Data Analysis'!$AB$2:$AB$23</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Data Analysis'!$B$1:$X$23</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Data Analysis'!$B$1:$X$23</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -1013,14 +1021,14 @@
         <v>3</v>
       </c>
       <c r="AG2" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH2" s="1">
         <v>3</v>
       </c>
       <c r="AI2" s="1">
         <f>SUM(AD2:AH2)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.2">
@@ -1127,14 +1135,14 @@
         <v>3</v>
       </c>
       <c r="AG3" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH3" s="1">
         <v>5</v>
       </c>
       <c r="AI3" s="1">
         <f>SUM(AD3:AH3)</f>
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.2">
@@ -1241,14 +1249,14 @@
         <v>3</v>
       </c>
       <c r="AG4" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH4" s="1">
         <v>3</v>
       </c>
       <c r="AI4" s="1">
         <f>SUM(AD4:AH4)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.2">
@@ -1352,7 +1360,7 @@
         <v>3</v>
       </c>
       <c r="AF5" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AG5" s="1">
         <v>5</v>
@@ -1362,7 +1370,7 @@
       </c>
       <c r="AI5" s="1">
         <f>SUM(AD5:AH5)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.2">
@@ -1583,14 +1591,14 @@
         <v>5</v>
       </c>
       <c r="AG7" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AH7" s="1">
         <v>3</v>
       </c>
       <c r="AI7" s="1">
         <f>SUM(AD7:AH7)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.2">
@@ -1697,14 +1705,14 @@
         <v>1</v>
       </c>
       <c r="AG8" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH8" s="1">
         <v>5</v>
       </c>
       <c r="AI8" s="1">
         <f>SUM(AD8:AH8)</f>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.2">
@@ -1811,14 +1819,14 @@
         <v>3</v>
       </c>
       <c r="AG9" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH9" s="1">
         <v>5</v>
       </c>
       <c r="AI9" s="1">
         <f>SUM(AD9:AH9)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.2">
@@ -1925,14 +1933,14 @@
         <v>1</v>
       </c>
       <c r="AG10" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH10" s="1">
         <v>4</v>
       </c>
       <c r="AI10" s="1">
         <f>SUM(AD10:AH10)</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.2">
@@ -2039,14 +2047,14 @@
         <v>3</v>
       </c>
       <c r="AG11" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AH11" s="1">
         <v>4</v>
       </c>
       <c r="AI11" s="1">
         <f>SUM(AD11:AH11)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.2">
@@ -2153,14 +2161,14 @@
         <v>1</v>
       </c>
       <c r="AG12" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH12" s="1">
         <v>5</v>
       </c>
       <c r="AI12" s="1">
         <f>SUM(AD12:AH12)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.2">
@@ -2267,14 +2275,14 @@
         <v>1</v>
       </c>
       <c r="AG13" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH13" s="1">
         <v>3</v>
       </c>
       <c r="AI13" s="1">
         <f>SUM(AD13:AH13)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.2">
@@ -2381,14 +2389,14 @@
         <v>1</v>
       </c>
       <c r="AG14" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH14" s="1">
         <v>5</v>
       </c>
       <c r="AI14" s="1">
         <f>SUM(AD14:AH14)</f>
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.2">
@@ -2495,14 +2503,14 @@
         <v>1</v>
       </c>
       <c r="AG15" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH15" s="1">
         <v>5</v>
       </c>
       <c r="AI15" s="1">
         <f>SUM(AD15:AH15)</f>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.2">
@@ -2606,7 +2614,7 @@
         <v>5</v>
       </c>
       <c r="AF16" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG16" s="1">
         <v>1</v>
@@ -2616,7 +2624,7 @@
       </c>
       <c r="AI16" s="1">
         <f>SUM(AD16:AH16)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.2">
@@ -2720,7 +2728,7 @@
         <v>5</v>
       </c>
       <c r="AF17" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG17" s="1">
         <v>1</v>
@@ -2730,7 +2738,7 @@
       </c>
       <c r="AI17" s="1">
         <f>SUM(AD17:AH17)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:35" x14ac:dyDescent="0.2">
@@ -2837,14 +2845,14 @@
         <v>1</v>
       </c>
       <c r="AG18" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH18" s="1">
         <v>5</v>
       </c>
       <c r="AI18" s="1">
         <f>SUM(AD18:AH18)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:35" x14ac:dyDescent="0.2">
@@ -2951,14 +2959,14 @@
         <v>2</v>
       </c>
       <c r="AG19" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH19" s="1">
         <v>5</v>
       </c>
       <c r="AI19" s="1">
         <f>SUM(AD19:AH19)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:35" x14ac:dyDescent="0.2">
@@ -3189,7 +3197,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:35" ht="10" x14ac:dyDescent="0.2">
       <c r="A22" t="str">
         <f>B22 &amp; " " &amp; C22</f>
         <v>ML-KEM  SPHINCS+</v>
@@ -3293,17 +3301,17 @@
         <v>1</v>
       </c>
       <c r="AG22" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH22" s="1">
         <v>5</v>
       </c>
       <c r="AI22" s="1">
         <f>SUM(AD22:AH22)</f>
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:35" ht="1" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
         <f>B23 &amp; " " &amp; C23</f>
         <v>ML-KEM  ML-DSA</v>
@@ -3416,6 +3424,18 @@
         <f>SUM(AD23:AH23)</f>
         <v>24</v>
       </c>
+    </row>
+    <row r="26" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Y26" s="1"/>
+      <c r="AB26" s="1"/>
+    </row>
+    <row r="27" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Y27" s="1"/>
+      <c r="AB27" s="1"/>
+    </row>
+    <row r="29" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Y29" s="1"/>
+      <c r="AB29" s="1"/>
     </row>
     <row r="30" spans="1:35" x14ac:dyDescent="0.2">
       <c r="E30" s="1"/>
@@ -3423,12 +3443,16 @@
       <c r="S30" s="1"/>
       <c r="U30" s="1"/>
       <c r="W30" s="1"/>
+      <c r="Y30" s="1"/>
+      <c r="AB30" s="1"/>
     </row>
     <row r="31" spans="1:35" x14ac:dyDescent="0.2">
       <c r="Q31" s="1"/>
       <c r="S31" s="1"/>
       <c r="U31" s="1"/>
       <c r="W31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="AB31" s="1"/>
     </row>
     <row r="32" spans="1:35" x14ac:dyDescent="0.2">
       <c r="E32" s="1"/>
@@ -3439,8 +3463,10 @@
       <c r="S32" s="1"/>
       <c r="U32" s="1"/>
       <c r="W32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="AB32" s="1"/>
     </row>
-    <row r="33" spans="5:23" x14ac:dyDescent="0.2">
+    <row r="33" spans="5:28" x14ac:dyDescent="0.2">
       <c r="E33" s="1"/>
       <c r="G33" s="1"/>
       <c r="I33" s="1"/>
@@ -3449,8 +3475,10 @@
       <c r="S33" s="1"/>
       <c r="U33" s="1"/>
       <c r="W33" s="1"/>
+      <c r="Y33" s="1"/>
+      <c r="AB33" s="1"/>
     </row>
-    <row r="34" spans="5:23" x14ac:dyDescent="0.2">
+    <row r="34" spans="5:28" x14ac:dyDescent="0.2">
       <c r="E34" s="1"/>
       <c r="G34" s="1"/>
       <c r="I34" s="1"/>

</xml_diff>